<commit_message>
updates years to include metadata
</commit_message>
<xml_diff>
--- a/data-raw/metadata/clear_years_to_include_metadata.xlsx
+++ b/data-raw/metadata/clear_years_to_include_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-clear-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE739190-CBD7-403C-94EF-0D633447BA30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C39D70-E7A4-49EB-898B-2462D65F9C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6400" yWindow="680" windowWidth="19200" windowHeight="11170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="attribute" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t xml:space="preserve">attribute_name </t>
   </si>
@@ -119,6 +119,12 @@
   </si>
   <si>
     <t>2024</t>
+  </si>
+  <si>
+    <t>data_type</t>
+  </si>
+  <si>
+    <t>Type of data collected. Levels = c("passage", redd")</t>
   </si>
 </sst>
 </file>
@@ -640,11 +646,21 @@
       <c r="Z4" s="7"/>
     </row>
     <row r="5" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="4"/>
+      <c r="A5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>

</xml_diff>